<commit_message>
Add end_date, building_type, military_installation, and amenity tags
end_date mirrors start_date (a year or DD/MM/YYYY date) for when something
ended rather than began. building_type classifies what kind of building a
point is (barn, house, hotel, store, and a dozen more common types) for
auto-fill from category/subcategory.

military_installation is the more involved one: most of its values name a
main installation's type (fort, castle, airbase, ...), but
military_installation_structure is a special value marking a secondary
building on such a site (a barracks, kitchen, mess hall, garage) rather
than naming an installation type. It combines with current (no longer
active vs. still standing) and the new amenity tag (starting with just
"museum") to distinguish a fort that's fallen entirely from one that still
stands and is now a museum.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UwnumY8psfaoQiTbhQ3ZB
</commit_message>
<xml_diff>
--- a/docs/point-tags/point-tags.xlsx
+++ b/docs/point-tags/point-tags.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -575,6 +575,102 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>YYYY;DD/MM/YYYY</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>building_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>barn;house;hotel;store;apartment;office;warehouse;garage;shed;cabin;church;school;hospital;factory;restaurant;library</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>military_installation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>military_installation_structure;fort;castle;airbase;base;camp;garrison;bunker;outpost</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>amenity</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>museum</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Promote military_installation_structure to its own tag
It was only a value of military_installation; now it's a second tag in its
own right, with values for what kind of secondary military building this
is (barracks, kitchen, mess hall, garage, and a few more). Tagging a
specific structure is a two-step handoff: military_installation:
military_installation_structure flags the point as some secondary building
on a military site, then this tag says exactly which kind.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UwnumY8psfaoQiTbhQ3ZB
</commit_message>
<xml_diff>
--- a/docs/point-tags/point-tags.xlsx
+++ b/docs/point-tags/point-tags.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -671,6 +671,30 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>military_installation_structure</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>barracks;kitchen;mess_hall;garage;armory;watchtower;gatehouse;infirmary;stable;guardhouse</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>